<commit_message>
feat: add simple implementation
</commit_message>
<xml_diff>
--- a/files/RFI-Examples.xlsx
+++ b/files/RFI-Examples.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Justine\MyFolder\File\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1FC3629F-2134-4A0B-B768-B3DB07D53DFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABBA1C50-7B6C-41D9-A450-6D7C7F1E4D0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{6F5E99A2-3C08-4B99-B702-F448B89F0FAF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{6F5E99A2-3C08-4B99-B702-F448B89F0FAF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="7">
   <si>
     <t>No</t>
   </si>
@@ -54,6 +55,9 @@
   </si>
   <si>
     <t>Yes/No</t>
+  </si>
+  <si>
+    <t>Why?</t>
   </si>
 </sst>
 </file>
@@ -477,4 +481,55 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E00EB6A6-E1A4-4B30-BD8C-8A09898E21DD}">
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="57.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>